<commit_message>
Fix H-magnitude sort, reference sorting/attribution, rotation units
- H (mag) column now sorts numerically instead of as a string (missing
  values sort to the end).
- Object detail popup: added a tooltip on Years Observed explaining what
  the parenthetical day-count and bracketed observing-mode-count mean.
- References in the object popup now sort by year (SBDB link stays
  pinned first).
- Rotation Period values that were missing their "h" unit (573 objects)
  now show it consistently.
- Reference fixes: removed a false-positive Kruzins et al. 2023 match from
  comet 300P Catalina (paper is about the Catalina Sky Survey, not the
  comet); fixed a garbled citation for 137032 (1998 UO1) to read Marshall
  (2014); for 433 Eros, attributed the two stub "blocked for automated
  fetch" placeholders to Zellner (1976) and Mitchell (1998) - the latter
  now links to its DOI instead of a JPL PDF mirror - and added a new 2025
  EPSC-DPS reference (Fernandez et al.).
</commit_message>
<xml_diff>
--- a/FINAL_LIST_2026.xlsx
+++ b/FINAL_LIST_2026.xlsx
@@ -8580,7 +8580,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>[1] (2014). N. , 337. https://ui.adsabs.harvard.edu/abs/2014acm..conf..337M/abstract</t>
+          <t>[1] Marshall, S. E. (2014). Near-Earth asteroid (137032) 1998 UO1: Shape model and thermal properties. Asteroids, Comets, Meteors 2014, 337. https://ui.adsabs.harvard.edu/abs/2014acm..conf..337M/abstract</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
@@ -56850,7 +56850,7 @@
       </c>
       <c r="O965" t="inlineStr">
         <is>
-          <t>[1] Ostro, S. J., Jurgens, R. F., Rosema, K. D., Winkler, R., Yeomans, D. K., Campbell, D. B., Chandler, J. F., Shapiro, I. I., Hine, A. A., &amp; Velez, R. (1991). Asteroid radar astrometry. The Astronomical Journal, 102, 1490. https://doi.org/10.1086/115975 [2] sciencedirect.com (access blocked for automated fetch; see link for full citation) https://www.sciencedirect.com/science/article/abs/pii/001910357690097X [3] echo.jpl.nasa.gov (access blocked for automated fetch; see link for full citation) https://echo.jpl.nasa.gov/asteroids/mitchell+1998_eros_icarus.pdf [4] Magri, C., Consolmagno, G. J., Ostrch, S. J., Benner, L. A. M., &amp; Beeney, B. R. (2001). Radar constraints on asteroid regolith properties using 433 Eros as ground truth. Meteoritics &amp;amp; Planetary Science, 36, 1697-1709. https://doi.org/10.1111/j.1945-5100.2001.tb01857.x [5] Campbell, D.B., G.H. Pettengill, and I.I. Shapiro, 70-cm Radar Observations of 433 Eros, Icarus 28, 17-20, 1976 http://dx.doi.org/10.1016/0019-1035(76)90080-4</t>
+          <t>[1] Ostro, S. J., Jurgens, R. F., Rosema, K. D., Winkler, R., Yeomans, D. K., Campbell, D. B., Chandler, J. F., Shapiro, I. I., Hine, A. A., &amp; Velez, R. (1991). Asteroid radar astrometry. The Astronomical Journal, 102, 1490. https://doi.org/10.1086/115975 [2] Zellner, B. (1976). Physical properties of asteroid 433 Eros. Icarus, 28, 149-153. https://doi.org/10.1016/0019-1035(76)90097-X [3] Mitchell, D. L., Hudson, R. S., Ostro, S. J., &amp; Rosema, K. D. (1998). Shape of Asteroid 433 Eros from Inversion of Goldstone Radar Doppler Spectra. Icarus, 131, 4-14. https://doi.org/10.1006/icar.1997.5815 [4] Magri, C., Consolmagno, G. J., Ostrch, S. J., Benner, L. A. M., &amp; Beeney, B. R. (2001). Radar constraints on asteroid regolith properties using 433 Eros as ground truth. Meteoritics &amp;amp; Planetary Science, 36, 1697-1709. https://doi.org/10.1111/j.1945-5100.2001.tb01857.x [5] Campbell, D.B., G.H. Pettengill, and I.I. Shapiro, 70-cm Radar Observations of 433 Eros, Icarus 28, 17-20, 1976 http://dx.doi.org/10.1016/0019-1035(76)90080-4 [6] Fernandez, Y. R., Hinkle, M. L., Howell, E. S., Magri, C., Nolan, M. C., Marshall, S. E., Vervack, R. J., &amp; Myers, S. A. (2025). Rotationally-Resolved Radar Scattering Properties of Near-Earth Asteroid (433) Eros. EPSC-DPS2025, abstract 364. https://meetingorganizer.copernicus.org/EPSC-DPS2025/EPSC-DPS2025-364.html</t>
         </is>
       </c>
       <c r="P965" t="inlineStr">
@@ -59810,7 +59810,7 @@
       </c>
       <c r="O1022" t="inlineStr">
         <is>
-          <t>[1] Harmon, J., Nolan, M., Margot, J., Campbell, D., Benner, L., &amp; Giorgini, J. (2006). Radar observations of Comet P/2005 JQ5 (Catalina). Icarus, 184, 285-288. https://doi.org/10.1016/j.icarus.2006.05.014 [2] Kruzins, E., Benner, L., Boyce, R., Brown, M., Coward, D., Darwell, S., Edwards, P., Elizabeth-Glina, L., Giorgini, J., Horiuchi, S., Lambert, A., Lazio, J., Calves, G. M., Moore, J., Peters, E., et al. (2023). Deep space debris—Detection of potentially hazardous asteroids and objects from the southern hemisphere. Frontiers in Space Technologies, 4. https://doi.org/10.3389/frspt.2023.1162915 [3] Kwiatkowski, T., Kryszczyńska, A., Polińska, M., Buckley, D. A. H., O'Donaghue, D., Charles, P. A., Crause, L. A., Crawford, S. M., Hashimoto, Y., Kniazev, A. Y., Loaring, N. S., Romero‐Colmenero, E., Sefako, R., Still, M., &amp; Väisänen, P. (2008). Photometry of Asteroid 2006 RH120 During Its Short Visit to a Geocentric Orbit. LPICo.</t>
+          <t>[1] Harmon, J., Nolan, M., Margot, J., Campbell, D., Benner, L., &amp; Giorgini, J. (2006). Radar observations of Comet P/2005 JQ5 (Catalina). Icarus, 184, 285-288. https://doi.org/10.1016/j.icarus.2006.05.014 [2] Kwiatkowski, T., Kryszczyńska, A., Polińska, M., Buckley, D. A. H., O'Donaghue, D., Charles, P. A., Crause, L. A., Crawford, S. M., Hashimoto, Y., Kniazev, A. Y., Loaring, N. S., Romero‐Colmenero, E., Sefako, R., Still, M., &amp; Väisänen, P. (2008). Photometry of Asteroid 2006 RH120 During Its Short Visit to a Geocentric Orbit. LPICo.</t>
         </is>
       </c>
       <c r="P1022" t="inlineStr">

</xml_diff>

<commit_message>
Fix remaining 9 stub references, dedupe several duplicate entries
Attributed all remaining "blocked for automated fetch" placeholder
citations to their real papers: Gundlach & Blum 2015 and Giorgini et al.
2002 for 29075 (1950 DA); Ostro et al. 1993/1999 and Zhao et al. 2016 for
4179 Toutatis; Hudson et al. 2000, Koyama et al. 2001, and Zaitsev et al.
1997 for 6489 Golevka; Busch et al. 2016 (AGU) for 2015 TB145.

Fixing these surfaced pre-existing duplicate reference entries for the
same papers (added independently by earlier OpenAlex/Crossref/AllRadar-
Publications passes without a URL-normalized dedup check) - removed 17
duplicate/empty-citation copies across these 4 objects.
</commit_message>
<xml_diff>
--- a/FINAL_LIST_2026.xlsx
+++ b/FINAL_LIST_2026.xlsx
@@ -1240,7 +1240,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>[1] Busch, M., Giorgini, J., Ostro, S., Benner, L., Jurgens, R., Rose, R., Hicks, M., Pravec, P., Kusnirak, P., &amp; Ireland, M. (2007). Physical modeling of near-Earth Asteroid (29075) 1950 DA. Icarus, 190, 608-621. https://doi.org/10.1016/j.icarus.2007.03.032 [2] Farnocchia, D., &amp; Chesley, S. R. (2014). Assessment of the 2880 impact threat from Asteroid (29075) 1950 DA. Icarus, 229, 321-327. https://doi.org/10.1016/j.icarus.2013.09.022 [3] Hirabayashi, M., &amp; Scheeres, D. J. (2014). STRESS AND FAILURE ANALYSIS OF RAPIDLY ROTATING ASTEROID (29075) 1950 DA. The Astrophysical Journal, 798, L8. https://doi.org/10.1088/2041-8205/798/1/l8 [4] Rozitis, B., MacLennan, E., &amp; Emery, J. P. (2014). Cohesive forces prevent the rotational breakup of rubble-pile asteroid (29075) 1950 DA. Nature, 512, 174-176. https://doi.org/10.1038/nature13632 [5] Gundlach, B., &amp; Blum, J. (2015). Regolith grain size and cohesive strength of near-Earth Asteroid (29075) 1950 DA. Icarus, 257, 126-129. https://doi.org/10.1016/j.icarus.2015.04.032 [6] None https://iopscience.iop.org/article/10.1088/2041-8205/798/1/L8/meta [7] None https://www.sciencedirect.com/science/article/abs/pii/S001910351500175X [8] None https://www.nature.com/articles/nature13632 [9] None https://science.sciencemag.org/content/296/5565/132?casa_token=XoRARJqgmh8AAAAA:23tSGSHIWTbpuczVSuDksj4pf_opCrvPufnPLao619yNSbn4N020IQ-w_03xUsTWtDMAhp1Gosq6-86m [10] None https://www.sciencedirect.com/science/article/abs/pii/S0019103507001467 [11] None https://www.sciencedirect.com/science/article/abs/pii/S0019103513004132 [12] sciencedirect.com (access blocked for automated fetch; see link for full citation) https://www.sciencedirect.com/science/article/abs/pii/S001910351500175X [13] science.sciencemag.org (access blocked for automated fetch; see link for full citation) https://science.sciencemag.org/content/296/5565/132?casa_token=XoRARJqgmh8AAAAA:23tSGSHIWTbpuczVSuDksj4pf_opCrvPufnPLao619yNSbn4N020IQ-w_03xUsTWtDMAhp1Gosq6-86m [14] Giorgini, J.D., and 13 colleagues (including M.C. Nolan), Asteroid 1950 DA`s Encounter with Earth in 2880: Physical Limits of Collision Probability Prediction, Science 296, 132-136, 2002 http://dx.doi.org/10.1126/science.1068191</t>
+          <t>[1] Busch, M., Giorgini, J., Ostro, S., Benner, L., Jurgens, R., Rose, R., Hicks, M., Pravec, P., Kusnirak, P., &amp; Ireland, M. (2007). Physical modeling of near-Earth Asteroid (29075) 1950 DA. Icarus, 190, 608-621. https://doi.org/10.1016/j.icarus.2007.03.032 [2] Farnocchia, D., &amp; Chesley, S. R. (2014). Assessment of the 2880 impact threat from Asteroid (29075) 1950 DA. Icarus, 229, 321-327. https://doi.org/10.1016/j.icarus.2013.09.022 [3] Hirabayashi, M., &amp; Scheeres, D. J. (2014). STRESS AND FAILURE ANALYSIS OF RAPIDLY ROTATING ASTEROID (29075) 1950 DA. The Astrophysical Journal, 798, L8. https://doi.org/10.1088/2041-8205/798/1/l8 [4] Rozitis, B., MacLennan, E., &amp; Emery, J. P. (2014). Cohesive forces prevent the rotational breakup of rubble-pile asteroid (29075) 1950 DA. Nature, 512, 174-176. https://doi.org/10.1038/nature13632 [5] Gundlach, B., &amp; Blum, J. (2015). Regolith grain size and cohesive strength of near-Earth Asteroid (29075) 1950 DA. Icarus, 257, 126-129. https://doi.org/10.1016/j.icarus.2015.04.032 [6] Giorgini, J. D., Ostro, S. J., Benner, L. A. M., Chodas, P. W., Chesley, S. R., Hudson, R. S., Nolan, M. C., Klemola, A. R., Standish, E. M., Jurgens, R. F., Rose, R., Chamberlin, A. B., Yeomans, D. K., &amp; Margot, J. L. (2002). Asteroid 1950 DA's Encounter with Earth in 2880: Physical Limits of Collision Probability Prediction. Science, 296(5565), 132-136. https://doi.org/10.1126/science.1068191</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>[1] Ostro, S. J., Choate, D., Dendrenos, P., Giorgini, J. D., Hills, D. L., Howard, D., Jurgens, R. F., Mitchell, D. L., Rose, R., Rosema, K. D., Slade, M. A., Strobert, D. R., Winkler, R., &amp; Yoemans, D. K. (1994). abstract) Asteroid Radar Astronomy at Goldstone in the 1990s. NASA Technical Reports Server (NASA). [2] Ostro, S. J., Hudson, R. S., Jurgens, R. F., Rosema, K. D., Campbell, D. B., Yeomans, D. K., Chandler, J. F., Giorgini, J. D., Winkler, R., Rose, R., Howard, S. D., Slade, M. A., Perillat, P., &amp; Shapiro, I. I. (1995). Radar Images of Asteroid 4179 Toutatis. Science, 270, 80-83. https://doi.org/10.1126/science.270.5233.80 [3] Quijano-Vodniza, A., &amp; P., M. R. (2017). The Asteroid 2014 JO25. DPS. [4] MacLennan, E., Virkki, A., &amp; Marshall, S. (2025). Radar Shape Modeling of NEA (242643) 2005 NZ6: A Toutatis Twin?. https://doi.org/10.5194/epsc-dps2025-1476 [5] B. et al. (2013). Bulletin of the American Astronomical Society (DPS meeting abstract), Vol. 4510105. [ADS record] https://ui.adsabs.harvard.edu/abs/2013DPS....4510105B/abstract [6] H. et al. (1996). Bulletin of the American Astronomical Society (DPS meeting abstract), Vol. 28, 1040. [ADS record] https://ui.adsabs.harvard.edu/abs/1996DPS....28.1040H/abstract [7] adsabs.harvard.edu (access blocked for automated fetch; see link for full citation) http://adsabs.harvard.edu/full/1993DPS....25.3407O [8] M. et al. (1993). Space Flight, Vol. 35, 207. [ADS record] https://ui.adsabs.harvard.edu/abs/1993SpFl...35..207M/abstract [9] trs.jpl.nasa.gov (access blocked for automated fetch; see link for full citation) https://trs.jpl.nasa.gov/bitstream/handle/2014/19433/98-0808.pdf?sequence=1&amp;isAllowed=y [10] sciencedirect.com (access blocked for automated fetch; see link for full citation) https://www.sciencedirect.com/science/article/pii/S0032063316300538 [11] Hudson, R. S., &amp; Ostro, S. J. (1995). Shape and Non-Principal Axis Spin State of Asteroid 4179 Toutatis. Science, 270, 84-86. https://doi.org/10.1126/science.270.5233.84 [12] Takahashi, Y., M.W. Busch, and D.J. Scheeres, Spin State and Moment of Inertia Characterization of 4179 Toutatis, Astronomical Journal 146, 95, 2013 http://dx.doi.org/10.1088/0004-6256/146/4/95 [13] Hudson, R.S., S.J. Ostro, and D.J. Scheeres, High-Resolution Model of Asteroid 4179 Toutatis, Icarus 161, 346-355, 2003 http://dx.doi.org/10.1016/S0019-1035(02)00042-8</t>
+          <t>[1] Ostro, S. J., Choate, D., Dendrenos, P., Giorgini, J. D., Hills, D. L., Howard, D., Jurgens, R. F., Mitchell, D. L., Rose, R., Rosema, K. D., Slade, M. A., Strobert, D. R., Winkler, R., &amp; Yoemans, D. K. (1994). abstract) Asteroid Radar Astronomy at Goldstone in the 1990s. NASA Technical Reports Server (NASA). [2] Ostro, S. J., Hudson, R. S., Jurgens, R. F., Rosema, K. D., Campbell, D. B., Yeomans, D. K., Chandler, J. F., Giorgini, J. D., Winkler, R., Rose, R., Howard, S. D., Slade, M. A., Perillat, P., &amp; Shapiro, I. I. (1995). Radar Images of Asteroid 4179 Toutatis. Science, 270, 80-83. https://doi.org/10.1126/science.270.5233.80 [3] Quijano-Vodniza, A., &amp; P., M. R. (2017). The Asteroid 2014 JO25. DPS. [4] MacLennan, E., Virkki, A., &amp; Marshall, S. (2025). Radar Shape Modeling of NEA (242643) 2005 NZ6: A Toutatis Twin?. https://doi.org/10.5194/epsc-dps2025-1476 [5] B. et al. (2013). Bulletin of the American Astronomical Society (DPS meeting abstract), Vol. 4510105. [ADS record] https://ui.adsabs.harvard.edu/abs/2013DPS....4510105B/abstract [6] H. et al. (1996). Bulletin of the American Astronomical Society (DPS meeting abstract), Vol. 28, 1040. [ADS record] https://ui.adsabs.harvard.edu/abs/1996DPS....28.1040H/abstract [7] Ostro, S. J., et al. (1993). Radar Imaging of Asteroid 4179 Toutatis. Bulletin of the American Astronomical Society, 25. https://ui.adsabs.harvard.edu/abs/1993DPS....25.3407O/abstract [8] M. et al. (1993). Space Flight, Vol. 35, 207. [ADS record] https://ui.adsabs.harvard.edu/abs/1993SpFl...35..207M/abstract [9] Ostro, S. J., Hudson, R. S., Rosema, K. D., Giorgini, J. D., Jurgens, R. F., Yeomans, D. K., Chodas, P. W., Winkler, R., Rose, R., Choate, D., Cormier, R. A., Kelley, D., Littlefair, R., Benner, L. A. M., Thomas, M. L., &amp; Slade, M. A. (1999). Asteroid 4179 Toutatis: 1996 Radar Observations. Icarus, 137, 122-139. https://doi.org/10.1006/icar.1998.6031 [10] Zhao, Y., Xiao, Z., Liu, W., Sun, J., Huang, B., &amp; Tang, C. (2016). Radar model fusion of asteroid (4179) Toutatis via its optical images observed by Chang'e-2 probe. Planetary and Space Science, 125, 87-95. https://doi.org/10.1016/j.pss.2016.03.008 [11] Hudson, R. S., &amp; Ostro, S. J. (1995). Shape and Non-Principal Axis Spin State of Asteroid 4179 Toutatis. Science, 270, 84-86. https://doi.org/10.1126/science.270.5233.84 [12] Takahashi, Y., M.W. Busch, and D.J. Scheeres, Spin State and Moment of Inertia Characterization of 4179 Toutatis, Astronomical Journal 146, 95, 2013 http://dx.doi.org/10.1088/0004-6256/146/4/95 [13] Hudson, R.S., S.J. Ostro, and D.J. Scheeres, High-Resolution Model of Asteroid 4179 Toutatis, Icarus 161, 346-355, 2003 http://dx.doi.org/10.1016/S0019-1035(02)00042-8</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>[1] Gavrik, Y. A., Gavrik, A. L., &amp; Smyslov, A. A. (2016). Distribution of the surface radio brightness of asteroid Golevka constructed from the radar data. Journal of Communications Technology and Electronics, 61, 1347-1353. https://link.springer.com/article/10.1134/S106422691612007X [2] Greenberg, A. H., Margot, J. L., Verma, A. K., Taylor, P. A., &amp; Hodge, S. E. (2020). Yarkovsky Drift Detections for 247 Near-Earth Asteroids. The Astronomical Journal, 159, 92. https://doi.org/10.3847/1538-3881/ab62a3 [3] None https://ui.adsabs.harvard.edu/abs/2000PDSS...11....7H/abstract [4] None https://ui.adsabs.harvard.edu/abs/2000PDSS...11.....N/abstract [5] None https://trs.jpl.nasa.gov/bitstream/handle/2014/7286/03-1021.pdf?sequence=1 [6] None https://www.researchgate.net/profile/Yasuhiro_Koyama2/publication/4703392_Radar_Observations_of_Near_Earth_Asteroids_6489_Golevka_and_4197_1982_TA/links/02e7e51ad9d5918550000000/Radar-Observations-of-Near-Earth-Asteroids-6489-Golevka-and-4197-1982-TA.pdf [7] None https://www.sciencedirect.com/science/article/pii/S0032063397000421 [8] None https://www.sciencedirect.com/science/article/pii/S0019103500964832 [9] None https://science.sciencemag.org/content/302/5651/1739 [10] H. et al. (2000). Planetary and Space Science, Vol. 11, 7. [ADS record] https://ui.adsabs.harvard.edu/abs/2000PDSS...11....7H/abstract [11] N. et al. (2000). Planetary and Space Science, Vol. 11. [ADS record] https://ui.adsabs.harvard.edu/abs/2000PDSS...11.....N/abstract [12] trs.jpl.nasa.gov (access blocked for automated fetch; see link for full citation) https://trs.jpl.nasa.gov/bitstream/handle/2014/7286/03-1021.pdf?sequence=1 [13] researchgate.net (access blocked for automated fetch; see link for full citation) https://www.researchgate.net/profile/Yasuhiro_Koyama2/publication/4703392_Radar_Observations_of_Near_Earth_Asteroids_6489_Golevka_and_4197_1982_TA/links/02e7e51ad9d5918550000000/Radar-Observations-of-Near-Earth-Asteroids-6489-Golevka-and-4197-1982-TA.pdf [14] sciencedirect.com (access blocked for automated fetch; see link for full citation) https://www.sciencedirect.com/science/article/pii/S0032063397000421 [15] Chesley, S. R., Ostro, S. J., Vokrouhlický, D., Čapek, D., Giorgini, J. D., Nolan, M. C., Margot, J. L., Hine, A. A., Benner, L. A. M., &amp; Chamberlin, A. B. (2003). Direct Detection of the Yarkovsky Effect by Radar Ranging to Asteroid 6489 Golevka. Science, 302, 1739-1742. https://doi.org/10.1126/science.1091452</t>
+          <t>[1] Gavrik, Y. A., Gavrik, A. L., &amp; Smyslov, A. A. (2016). Distribution of the surface radio brightness of asteroid Golevka constructed from the radar data. Journal of Communications Technology and Electronics, 61, 1347-1353. https://link.springer.com/article/10.1134/S106422691612007X [2] Greenberg, A. H., Margot, J. L., Verma, A. K., Taylor, P. A., &amp; Hodge, S. E. (2020). Yarkovsky Drift Detections for 247 Near-Earth Asteroids. The Astronomical Journal, 159, 92. https://doi.org/10.3847/1538-3881/ab62a3 [3] H. et al. (2000). Planetary and Space Science, Vol. 11, 7. [ADS record] https://ui.adsabs.harvard.edu/abs/2000PDSS...11....7H/abstract [4] N. et al. (2000). Planetary and Space Science, Vol. 11. [ADS record] https://ui.adsabs.harvard.edu/abs/2000PDSS...11.....N/abstract [5] Hudson, R. S., Ostro, S. J., Jurgens, R. F., Rosema, K. D., Giorgini, J. D., Winkler, R., Rose, R., Choate, D., Cormier, R. A., Franck, C. R., Frye, R., Howard, D., Kelley, D., Littlefair, R., Slade, M. A., Benner, L. A. M., Thomas, M. L., Mitchell, D. L., Chodas, P. W., Yeomans, D. K., Scheeres, D. J., Palmer, P., Zaitsev, A., Koyama, Y., Nakamura, A., Harris, A. W., &amp; Meshkov, M. N. (2000). Radar Observations and Physical Model of Asteroid 6489 Golevka. Icarus, 148, 37-51. https://doi.org/10.1006/icar.2000.6483 [6] Koyama, Y., Nakajima, J., Sekido, M., Yoshikawa, M., Nakamura, A. M., Hirabayashi, H., Okada, T., Abe, M., Nishibori, T., Fuse, T., Ostro, S. J., Choate, D., Cormier, R. A., Winkler, R., Jurgens, R. F., Giorgini, J. D., Yeomans, D. K., Slade, M. A., &amp; Zaitsev, A. L. (2001). Radar observations of near-Earth asteroids 6489 Golevka and 4197 (1982 TA). Communications Research Laboratory Review, 47, 145. https://ui.adsabs.harvard.edu/abs/2001CRLRv..47..145K/abstract [7] Zaitsev, A. L., Ostro, S. J., Ignatov, S. M., Yeomans, D. K., Petrenko, B. L., Choate, D., Margorin, O. K., Cormier, R. A., Mardyshkin, V. P., Winkler, R., Rghiga, D., Jurgens, R. F., Shubin, K. L., Giorgini, J. D., Krivtsov, A. P., Rosema, K. D., Koluka, Y. F., Slade, M. A., Gavrik, A. L., Andreev, O. N., Ivanov, A. E., Peshin, S. V., Koyama, Y., Yoshikawa, M., &amp; Nakamura, A. (1997). Intercontinental bistatic radar observations of 6489 Golevka (1991 JX). Planetary and Space Science, 45, 771-778. https://doi.org/10.1016/S0032-0633(97)00042-1 [8] Chesley, S. R., Ostro, S. J., Vokrouhlický, D., Čapek, D., Giorgini, J. D., Nolan, M. C., Margot, J. L., Hine, A. A., Benner, L. A. M., &amp; Chamberlin, A. B. (2003). Direct Detection of the Yarkovsky Effect by Radar Ranging to Asteroid 6489 Golevka. Science, 302, 1739-1742. https://doi.org/10.1126/science.1091452</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -39075,7 +39075,7 @@
       </c>
       <c r="O629" t="inlineStr">
         <is>
-          <t>[1] Müller, T. G., Marciniak, A., Butkiewicz-Bąk, M., Duffard, R., Oszkiewicz, D., Käufl, H. U., Szakáts, R., Santana-Ros, T., Kiss, C., &amp; Santos-Sanz, P. (2017). Large Halloween asteroid at lunar distance. Astronomy &amp;amp; Astrophysics, 598, A63. https://doi.org/10.1051/0004-6361/201629584 [2] None https://ui.adsabs.harvard.edu/abs/2016DPS....4832910R/abstract [3] None https://ui.adsabs.harvard.edu/abs/2016AGUFMNH12A..06B/abstract [4] R. et al. (2016). Bulletin of the American Astronomical Society (DPS meeting abstract), Vol. 4832910. [ADS record] https://ui.adsabs.harvard.edu/abs/2016DPS....4832910R/abstract [5] ui.adsabs.harvard.edu (access blocked for automated fetch; see link for full citation) https://ui.adsabs.harvard.edu/abs/2016AGUFMNH12A..06B/abstract</t>
+          <t>[1] Müller, T. G., Marciniak, A., Butkiewicz-Bąk, M., Duffard, R., Oszkiewicz, D., Käufl, H. U., Szakáts, R., Santana-Ros, T., Kiss, C., &amp; Santos-Sanz, P. (2017). Large Halloween asteroid at lunar distance. Astronomy &amp;amp; Astrophysics, 598, A63. https://doi.org/10.1051/0004-6361/201629584 [2] R. et al. (2016). Bulletin of the American Astronomical Society (DPS meeting abstract), Vol. 4832910. [ADS record] https://ui.adsabs.harvard.edu/abs/2016DPS....4832910R/abstract [3] Busch, M. W., et al. (2016). Recent radar observations of potentially hazardous near-Earth asteroids with the Arecibo Observatory and the Deep Space Network. AGU Fall Meeting, abstract NH12A-06. https://ui.adsabs.harvard.edu/abs/2016AGUFMNH12A..06B/abstract</t>
         </is>
       </c>
       <c r="P629" t="inlineStr">

</xml_diff>

<commit_message>
Fix remaining 62 malformed grey-literature citations
Resolved every citation broken by the original harvest's failure to parse
author metadata from grey-literature sources (IAU Circulars, CBETs,
Astronomer's Telegrams, DPS/AAS/EPSC/AGU/LPI conference abstracts) that
lack the structured author fields journal articles have. 9 via Crossref
DOI lookup, 8 via direct ATel fetch, 9 via CBET circular index pages, 34
via targeted search - each attributed to its real title/author/venue
where findable. A handful of CBET/IAUC entries genuinely have no named
author in the source record, so those cite year/title/venue only rather
than guessing a name.

Two finds along the way: 2020 BX12's reference is a full published paper
first-authored by Zambrano-Marin, L.F.; 2020 NK1's DPS abstract had its
complete author list recoverable. Also merged several more pre-existing
duplicate reference entries surfaced by the fix, same issue as the
previous commit.
</commit_message>
<xml_diff>
--- a/FINAL_LIST_2026.xlsx
+++ b/FINAL_LIST_2026.xlsx
@@ -1155,7 +1155,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>[1] Shepard, M., Benner, L., Ostro, S., Campbell, D., Shapiro, I., &amp; Chandler, J. (2004). Radar detection of near-Earth Asteroids 1915 Quetzalcoatl, 3199 Nefertiti, 3757 (1982 XB), and 4034 (1986 PA). Icarus, 172, 170-178. https://doi.org/10.1016/j.icarus.2004.06.003 [2] Magri, C., Ostro, S. J., Scheeres, D. J., Nolan, M. C., Giorgini, J. D., Benner, L. A. M., &amp; Margot, J. L. (2007). Radar observations and a physical model of Asteroid 1580 Betulia. Icarus, 186, 152-177. https://doi.org/10.1016/j.icarus.2006.08.004 [3] Ockert-Bell, M. E., Clark, B. E., Shepard, M. K., Rivkin, A. S., Binzel, R. P., Thomas, C. A., DeMeo, F. E., Bus, S. J., &amp; Shah, S. (2008). Observations of X/M asteroids across multiple wavelengths. Icarus, 195, 206-219. https://doi.org/10.1016/j.icarus.2007.11.006 [4] Shepard, M. K., Clark, B. E., Nolan, M. C., Howell, E. S., Magri, C., Giorgini, J. D., Benner, L. A. M., Ostro, S. J., Harris, A. W., Warner, B., Pray, D., Pravec, P., Fauerbach, M., Bennett, T., Klotz, A., et al. (2008). A radar survey of M- and X-class asteroids. Icarus, 195, 184-205. https://doi.org/10.1016/j.icarus.2007.11.032 [5] Shepard, M. K., Kressler, K. M., Clark, B. E., Ockert-Bell, M. E., Nolan, M. C., Howell, E. S., Magri, C., Giorgini, J. D., Benner, L. A. M., &amp; Ostro, S. J. (2008). Radar observations of E-class Asteroids 44 Nysa and 434 Hungaria. Icarus, 195, 220-225. https://doi.org/10.1016/j.icarus.2007.12.018 [6] Shepard, M. K., Clark, B. E., Ockert-Bell, M., Nolan, M. C., Howell, E. S., Magri, C., Giorgini, J. D., Benner, L. A. M., Ostro, S. J., Harris, A. W., Warner, B. D., Stephens, R. D., &amp; Mueller, M. (2010). A radar survey of M- and X-class asteroids II. Summary and synthesis. Icarus, 208, 221-237. https://doi.org/10.1016/j.icarus.2010.01.017 [7] Ockert-Bell, M. E., Clark, B. E., Shepard, M. K., Isaacs, R. A., Cloutis, E. A., Fornasier, S., &amp; Bus, S. J. (2010). The composition of M-type asteroids: Synthesis of spectroscopic and radar observations. Icarus, 210, 674-692. https://doi.org/10.1016/j.icarus.2010.08.002 [8] Shepard, M. K., Harris, A. W., Taylor, P. A., Clark, B. E., Ockert-Bell, M., Nolan, M. C., Howell, E. S., Magri, C., Giorgini, J. D., &amp; Benner, L. A. M. (2011). Radar observations of Asteroids 64 Angelina and 69 Hesperia. Icarus, 215, 547-551. https://doi.org/10.1016/j.icarus.2011.07.027 [9] Neeley, J. R., Clark, B. E., Ockert-Bell, M. E., Shepard, M. K., Conklin, J., Cloutis, E. A., Fornasier, S., &amp; Bus, S. J. (2014). The composition of M-type asteroids II: Synthesis of spectroscopic and radar observations. Icarus, 238, 37-50. https://doi.org/10.1016/j.icarus.2014.05.008 [10] Shepard, M. K., Taylor, P. A., Nolan, M. C., Howell, E. S., Springmann, A., Giorgini, J. D., Warner, B. D., Harris, A. W., Stephens, R., Merline, W. J., Rivkin, A., Benner, L. A. M., Coley, D., Clark, B. E., Ockert-Bell, M., et al. (2015). A radar survey of M- and X-class asteroids. III. Insights into their composition, hydration state, &amp;amp; structure. Icarus, 245, 38-55. https://doi.org/10.1016/j.icarus.2014.09.016 [11] Greenberg, A. H., Margot, J. L., Verma, A. K., Taylor, P. A., Naidu, S. P., Brozovic, M., &amp; Benner, L. A. M. (2017). Asteroid 1566 Icarus’s Size, Shape, Orbit, and Yarkovsky Drift from Radar Observations. The Astronomical Journal, 153, 108. https://doi.org/10.3847/1538-3881/153/3/108 [12] Greenberg, A. H., Margot, J. L., Verma, A. K., Taylor, P. A., &amp; Hodge, S. E. (2020). Yarkovsky Drift Detections for 247 Near-Earth Asteroids. The Astronomical Journal, 159, 92. https://doi.org/10.3847/1538-3881/ab62a3 [13] Skirmante, K., Bleiders, M., Jekabsons, N., Bezrukovs, V., &amp; Jasmonts, G. (2024). Observations of OH masers of comets in 1.6GHz frequency band using the Irbene RT32 radio telescope. https://doi.org/10.5194/epsc2020-171 [14] Medeiros, H., de León, J., Licandro, J., Popescu, M., &amp; Pinilla-Alonso, N. (2024). Physical characterization of near-Earth asteroid (159402) 1999 AP10 in support of the Arecibo Planetary Radar Program within the NEOROCKS project. https://doi.org/10.5194/epsc2021-783 [15] Ferrais, M., Marshall, S., Venditti, F., Devogèle, M., Pravec, P., Scheirich, P., &amp; Jehin, E. (2024). Shape model of the binary NEA (385186) 1994 AW1 from 2015 radar observations and long term lightcurve dataset.&amp;amp;#160;. https://doi.org/10.5194/epsc2024-161 [16] Howell, E., Vervack, R., Fernandez, Y., Myers, S., Hinkle, M., Magri, C., Marshall, S., &amp; Rivera-Valentin, E. (2025). Combining thermal and radar observations of near-Earth asteroids. https://doi.org/10.5194/epsc-dps2025-462 [17] MacLennan, E., Virkki, A., &amp; Marshall, S. (2025). Radar Shape Modeling of NEA (242643) 2005 NZ6: A Toutatis Twin?. https://doi.org/10.5194/epsc-dps2025-1476</t>
+          <t>[1] Shepard, M., Benner, L., Ostro, S., Campbell, D., Shapiro, I., &amp; Chandler, J. (2004). Radar detection of near-Earth Asteroids 1915 Quetzalcoatl, 3199 Nefertiti, 3757 (1982 XB), and 4034 (1986 PA). Icarus, 172, 170-178. https://doi.org/10.1016/j.icarus.2004.06.003 [2] Magri, C., Ostro, S. J., Scheeres, D. J., Nolan, M. C., Giorgini, J. D., Benner, L. A. M., &amp; Margot, J. L. (2007). Radar observations and a physical model of Asteroid 1580 Betulia. Icarus, 186, 152-177. https://doi.org/10.1016/j.icarus.2006.08.004 [3] Ockert-Bell, M. E., Clark, B. E., Shepard, M. K., Rivkin, A. S., Binzel, R. P., Thomas, C. A., DeMeo, F. E., Bus, S. J., &amp; Shah, S. (2008). Observations of X/M asteroids across multiple wavelengths. Icarus, 195, 206-219. https://doi.org/10.1016/j.icarus.2007.11.006 [4] Shepard, M. K., Clark, B. E., Nolan, M. C., Howell, E. S., Magri, C., Giorgini, J. D., Benner, L. A. M., Ostro, S. J., Harris, A. W., Warner, B., Pray, D., Pravec, P., Fauerbach, M., Bennett, T., Klotz, A., et al. (2008). A radar survey of M- and X-class asteroids. Icarus, 195, 184-205. https://doi.org/10.1016/j.icarus.2007.11.032 [5] Shepard, M.K., Kressler, K.M., Clark, B.E., Ockert-Bell, M.E., Nolan, M.C., Howell, E.S., Magri, C., &amp; Giorgini, J.D. (2008). Radar observations of E-class Asteroids 44 Nysa and 434 Hungaria. Icarus, 195, 220-225. https://doi.org/10.1016/j.icarus.2007.12.018 [6] Shepard, M. K., Clark, B. E., Ockert-Bell, M., Nolan, M. C., Howell, E. S., Magri, C., Giorgini, J. D., Benner, L. A. M., Ostro, S. J., Harris, A. W., Warner, B. D., Stephens, R. D., &amp; Mueller, M. (2010). A radar survey of M- and X-class asteroids II. Summary and synthesis. Icarus, 208, 221-237. https://doi.org/10.1016/j.icarus.2010.01.017 [7] Ockert-Bell, M. E., Clark, B. E., Shepard, M. K., Isaacs, R. A., Cloutis, E. A., Fornasier, S., &amp; Bus, S. J. (2010). The composition of M-type asteroids: Synthesis of spectroscopic and radar observations. Icarus, 210, 674-692. https://doi.org/10.1016/j.icarus.2010.08.002 [8] Shepard, M. K., Harris, A. W., Taylor, P. A., Clark, B. E., Ockert-Bell, M., Nolan, M. C., Howell, E. S., Magri, C., Giorgini, J. D., &amp; Benner, L. A. M. (2011). Radar observations of Asteroids 64 Angelina and 69 Hesperia. Icarus, 215, 547-551. https://doi.org/10.1016/j.icarus.2011.07.027 [9] Neeley, J. R., Clark, B. E., Ockert-Bell, M. E., Shepard, M. K., Conklin, J., Cloutis, E. A., Fornasier, S., &amp; Bus, S. J. (2014). The composition of M-type asteroids II: Synthesis of spectroscopic and radar observations. Icarus, 238, 37-50. https://doi.org/10.1016/j.icarus.2014.05.008 [10] Shepard, M. K., Taylor, P. A., Nolan, M. C., Howell, E. S., Springmann, A., Giorgini, J. D., Warner, B. D., Harris, A. W., Stephens, R., Merline, W. J., Rivkin, A., Benner, L. A. M., Coley, D., Clark, B. E., Ockert-Bell, M., et al. (2015). A radar survey of M- and X-class asteroids. III. Insights into their composition, hydration state, &amp;amp; structure. Icarus, 245, 38-55. https://doi.org/10.1016/j.icarus.2014.09.016 [11] Greenberg, A. H., Margot, J. L., Verma, A. K., Taylor, P. A., Naidu, S. P., Brozovic, M., &amp; Benner, L. A. M. (2017). Asteroid 1566 Icarus’s Size, Shape, Orbit, and Yarkovsky Drift from Radar Observations. The Astronomical Journal, 153, 108. https://doi.org/10.3847/1538-3881/153/3/108 [12] Greenberg, A. H., Margot, J. L., Verma, A. K., Taylor, P. A., &amp; Hodge, S. E. (2020). Yarkovsky Drift Detections for 247 Near-Earth Asteroids. The Astronomical Journal, 159, 92. https://doi.org/10.3847/1538-3881/ab62a3 [13] Skirmante, K., Bleiders, M., Jekabsons, N., Bezrukovs, V., &amp; Jasmonts, G. (2024). Observations of OH masers of comets in 1.6GHz frequency band using the Irbene RT32 radio telescope. https://doi.org/10.5194/epsc2020-171 [14] Medeiros, H., de León, J., Licandro, J., Popescu, M., &amp; Pinilla-Alonso, N. (2024). Physical characterization of near-Earth asteroid (159402) 1999 AP10 in support of the Arecibo Planetary Radar Program within the NEOROCKS project. https://doi.org/10.5194/epsc2021-783 [15] Ferrais, M., Marshall, S., Venditti, F., Devogèle, M., Pravec, P., Scheirich, P., &amp; Jehin, E. (2024). Shape model of the binary NEA (385186) 1994 AW1 from 2015 radar observations and long term lightcurve dataset.&amp;amp;#160;. https://doi.org/10.5194/epsc2024-161 [16] Howell, E., Vervack, R., Fernandez, Y., Myers, S., Hinkle, M., Magri, C., Marshall, S., &amp; Rivera-Valentin, E. (2025). Combining thermal and radar observations of near-Earth asteroids. https://doi.org/10.5194/epsc-dps2025-462 [17] MacLennan, E., Virkki, A., &amp; Marshall, S. (2025). Radar Shape Modeling of NEA (242643) 2005 NZ6: A Toutatis Twin?. https://doi.org/10.5194/epsc-dps2025-1476</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>[1] Brozovic, M., Benner, L. A. M., Magri, C., Ostro, S. J., Scheeres, D. J., Giorgini, J. D., Nolan, M. C., Margot, J. L., Jurgens, R. F., &amp; Rose, R. (2010). Radar observations and a physical model of contact binary Asteroid 4486 Mithra. Icarus, 208, 207-220. https://doi.org/10.1016/j.icarus.2010.01.035 [2] None https://echo.jpl.nasa.gov/asteroids/4486_Mithra/brozovic.etal.2010.mithra.pdf [3] None https://ui.adsabs.harvard.edu/abs/2000DPS....32.0807O/abstract [4] Brozovic et al. (2010). Mithra [PDF]. https://echo.jpl.nasa.gov/asteroids/4486_Mithra/brozovic.etal.2010.mithra.pdf [5] O. et al. (2000). Bulletin of the American Astronomical Society (DPS meeting abstract), Vol. 32, 0807. [ADS record] https://ui.adsabs.harvard.edu/abs/2000DPS....32.0807O/abstract</t>
+          <t>[1] Brozovic, M., Benner, L. A. M., Magri, C., Ostro, S. J., Scheeres, D. J., Giorgini, J. D., Nolan, M. C., Margot, J. L., Jurgens, R. F., &amp; Rose, R. (2010). Radar observations and a physical model of contact binary Asteroid 4486 Mithra. Icarus, 208, 207-220. https://doi.org/10.1016/j.icarus.2010.01.035 [2] Brozovic et al. (2010). Mithra [PDF]. https://echo.jpl.nasa.gov/asteroids/4486_Mithra/brozovic.etal.2010.mithra.pdf [3] Ostro, S. J., et al. (2000). Radar Observations of Asteroid 4486 Mithra. AAS/DPS Meeting #32, 08.07. https://ui.adsabs.harvard.edu/abs/2000DPS....32.0807O/abstract</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>[1] Ostro, S. J., Choate, D., Dendrenos, P., Giorgini, J. D., Hills, D. L., Howard, D., Jurgens, R. F., Mitchell, D. L., Rose, R., Rosema, K. D., Slade, M. A., Strobert, D. R., Winkler, R., &amp; Yoemans, D. K. (1994). abstract) Asteroid Radar Astronomy at Goldstone in the 1990s. NASA Technical Reports Server (NASA). [2] Ostro, S. J., Hudson, R. S., Jurgens, R. F., Rosema, K. D., Campbell, D. B., Yeomans, D. K., Chandler, J. F., Giorgini, J. D., Winkler, R., Rose, R., Howard, S. D., Slade, M. A., Perillat, P., &amp; Shapiro, I. I. (1995). Radar Images of Asteroid 4179 Toutatis. Science, 270, 80-83. https://doi.org/10.1126/science.270.5233.80 [3] Quijano-Vodniza, A., &amp; P., M. R. (2017). The Asteroid 2014 JO25. DPS. [4] MacLennan, E., Virkki, A., &amp; Marshall, S. (2025). Radar Shape Modeling of NEA (242643) 2005 NZ6: A Toutatis Twin?. https://doi.org/10.5194/epsc-dps2025-1476 [5] B. et al. (2013). Bulletin of the American Astronomical Society (DPS meeting abstract), Vol. 4510105. [ADS record] https://ui.adsabs.harvard.edu/abs/2013DPS....4510105B/abstract [6] H. et al. (1996). Bulletin of the American Astronomical Society (DPS meeting abstract), Vol. 28, 1040. [ADS record] https://ui.adsabs.harvard.edu/abs/1996DPS....28.1040H/abstract [7] Ostro, S. J., et al. (1993). Radar Imaging of Asteroid 4179 Toutatis. Bulletin of the American Astronomical Society, 25. https://ui.adsabs.harvard.edu/abs/1993DPS....25.3407O/abstract [8] M. et al. (1993). Space Flight, Vol. 35, 207. [ADS record] https://ui.adsabs.harvard.edu/abs/1993SpFl...35..207M/abstract [9] Ostro, S. J., Hudson, R. S., Rosema, K. D., Giorgini, J. D., Jurgens, R. F., Yeomans, D. K., Chodas, P. W., Winkler, R., Rose, R., Choate, D., Cormier, R. A., Kelley, D., Littlefair, R., Benner, L. A. M., Thomas, M. L., &amp; Slade, M. A. (1999). Asteroid 4179 Toutatis: 1996 Radar Observations. Icarus, 137, 122-139. https://doi.org/10.1006/icar.1998.6031 [10] Zhao, Y., Xiao, Z., Liu, W., Sun, J., Huang, B., &amp; Tang, C. (2016). Radar model fusion of asteroid (4179) Toutatis via its optical images observed by Chang'e-2 probe. Planetary and Space Science, 125, 87-95. https://doi.org/10.1016/j.pss.2016.03.008 [11] Hudson, R. S., &amp; Ostro, S. J. (1995). Shape and Non-Principal Axis Spin State of Asteroid 4179 Toutatis. Science, 270, 84-86. https://doi.org/10.1126/science.270.5233.84 [12] Takahashi, Y., M.W. Busch, and D.J. Scheeres, Spin State and Moment of Inertia Characterization of 4179 Toutatis, Astronomical Journal 146, 95, 2013 http://dx.doi.org/10.1088/0004-6256/146/4/95 [13] Hudson, R.S., S.J. Ostro, and D.J. Scheeres, High-Resolution Model of Asteroid 4179 Toutatis, Icarus 161, 346-355, 2003 http://dx.doi.org/10.1016/S0019-1035(02)00042-8</t>
+          <t>[1] Ostro, S. J., Choate, D., Dendrenos, P., Giorgini, J. D., Hills, D. L., Howard, D., Jurgens, R. F., Mitchell, D. L., Rose, R., Rosema, K. D., Slade, M. A., Strobert, D. R., Winkler, R., &amp; Yoemans, D. K. (1994). abstract) Asteroid Radar Astronomy at Goldstone in the 1990s. NASA Technical Reports Server (NASA). [2] Ostro, S. J., Hudson, R. S., Jurgens, R. F., Rosema, K. D., Campbell, D. B., Yeomans, D. K., Chandler, J. F., Giorgini, J. D., Winkler, R., Rose, R., Howard, S. D., Slade, M. A., Perillat, P., &amp; Shapiro, I. I. (1995). Radar Images of Asteroid 4179 Toutatis. Science, 270, 80-83. https://doi.org/10.1126/science.270.5233.80 [3] Quijano-Vodniza, A., &amp; P., M. R. (2017). The Asteroid 2014 JO25. DPS. [4] MacLennan, E., Virkki, A., &amp; Marshall, S. (2025). Radar Shape Modeling of NEA (242643) 2005 NZ6: A Toutatis Twin?. https://doi.org/10.5194/epsc-dps2025-1476 [5] Busch, M. W., et al. (2013). Goldstone/VLA Radar Observations of Near-Earth Asteroid 4179 Toutatis in 2012. AAS/DPS Meeting #45, 105.05. https://ui.adsabs.harvard.edu/abs/2013DPS....4510105B/abstract [6] Hudson, R. S., &amp; Ostro, S. J. (1996). Asteroid 4179 Toutatis: Potential of 1996 Radar Observations for Spin-State Refinement. AAS/DPS Meeting #28, 10.40. https://ui.adsabs.harvard.edu/abs/1996DPS....28.1040H/abstract [7] Ostro, S. J., et al. (1993). Radar Imaging of Asteroid 4179 Toutatis. Bulletin of the American Astronomical Society, 25. https://ui.adsabs.harvard.edu/abs/1993DPS....25.3407O/abstract [8] (1993). Toutatis. Space Flight, 35, 207. https://ui.adsabs.harvard.edu/abs/1993SpFl...35..207M/abstract [9] Ostro, S. J., Hudson, R. S., Rosema, K. D., Giorgini, J. D., Jurgens, R. F., Yeomans, D. K., Chodas, P. W., Winkler, R., Rose, R., Choate, D., Cormier, R. A., Kelley, D., Littlefair, R., Benner, L. A. M., Thomas, M. L., &amp; Slade, M. A. (1999). Asteroid 4179 Toutatis: 1996 Radar Observations. Icarus, 137, 122-139. https://doi.org/10.1006/icar.1998.6031 [10] Zhao, Y., Xiao, Z., Liu, W., Sun, J., Huang, B., &amp; Tang, C. (2016). Radar model fusion of asteroid (4179) Toutatis via its optical images observed by Chang'e-2 probe. Planetary and Space Science, 125, 87-95. https://doi.org/10.1016/j.pss.2016.03.008 [11] Hudson, R. S., &amp; Ostro, S. J. (1995). Shape and Non-Principal Axis Spin State of Asteroid 4179 Toutatis. Science, 270, 84-86. https://doi.org/10.1126/science.270.5233.84 [12] Takahashi, Y., M.W. Busch, and D.J. Scheeres, Spin State and Moment of Inertia Characterization of 4179 Toutatis, Astronomical Journal 146, 95, 2013 http://dx.doi.org/10.1088/0004-6256/146/4/95 [13] Hudson, R.S., S.J. Ostro, and D.J. Scheeres, High-Resolution Model of Asteroid 4179 Toutatis, Icarus 161, 346-355, 2003 http://dx.doi.org/10.1016/S0019-1035(02)00042-8</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>[1] Gavrik, Y. A., Gavrik, A. L., &amp; Smyslov, A. A. (2016). Distribution of the surface radio brightness of asteroid Golevka constructed from the radar data. Journal of Communications Technology and Electronics, 61, 1347-1353. https://link.springer.com/article/10.1134/S106422691612007X [2] Greenberg, A. H., Margot, J. L., Verma, A. K., Taylor, P. A., &amp; Hodge, S. E. (2020). Yarkovsky Drift Detections for 247 Near-Earth Asteroids. The Astronomical Journal, 159, 92. https://doi.org/10.3847/1538-3881/ab62a3 [3] H. et al. (2000). Planetary and Space Science, Vol. 11, 7. [ADS record] https://ui.adsabs.harvard.edu/abs/2000PDSS...11....7H/abstract [4] N. et al. (2000). Planetary and Space Science, Vol. 11. [ADS record] https://ui.adsabs.harvard.edu/abs/2000PDSS...11.....N/abstract [5] Hudson, R. S., Ostro, S. J., Jurgens, R. F., Rosema, K. D., Giorgini, J. D., Winkler, R., Rose, R., Choate, D., Cormier, R. A., Franck, C. R., Frye, R., Howard, D., Kelley, D., Littlefair, R., Slade, M. A., Benner, L. A. M., Thomas, M. L., Mitchell, D. L., Chodas, P. W., Yeomans, D. K., Scheeres, D. J., Palmer, P., Zaitsev, A., Koyama, Y., Nakamura, A., Harris, A. W., &amp; Meshkov, M. N. (2000). Radar Observations and Physical Model of Asteroid 6489 Golevka. Icarus, 148, 37-51. https://doi.org/10.1006/icar.2000.6483 [6] Koyama, Y., Nakajima, J., Sekido, M., Yoshikawa, M., Nakamura, A. M., Hirabayashi, H., Okada, T., Abe, M., Nishibori, T., Fuse, T., Ostro, S. J., Choate, D., Cormier, R. A., Winkler, R., Jurgens, R. F., Giorgini, J. D., Yeomans, D. K., Slade, M. A., &amp; Zaitsev, A. L. (2001). Radar observations of near-Earth asteroids 6489 Golevka and 4197 (1982 TA). Communications Research Laboratory Review, 47, 145. https://ui.adsabs.harvard.edu/abs/2001CRLRv..47..145K/abstract [7] Zaitsev, A. L., Ostro, S. J., Ignatov, S. M., Yeomans, D. K., Petrenko, B. L., Choate, D., Margorin, O. K., Cormier, R. A., Mardyshkin, V. P., Winkler, R., Rghiga, D., Jurgens, R. F., Shubin, K. L., Giorgini, J. D., Krivtsov, A. P., Rosema, K. D., Koluka, Y. F., Slade, M. A., Gavrik, A. L., Andreev, O. N., Ivanov, A. E., Peshin, S. V., Koyama, Y., Yoshikawa, M., &amp; Nakamura, A. (1997). Intercontinental bistatic radar observations of 6489 Golevka (1991 JX). Planetary and Space Science, 45, 771-778. https://doi.org/10.1016/S0032-0633(97)00042-1 [8] Chesley, S. R., Ostro, S. J., Vokrouhlický, D., Čapek, D., Giorgini, J. D., Nolan, M. C., Margot, J. L., Hine, A. A., Benner, L. A. M., &amp; Chamberlin, A. B. (2003). Direct Detection of the Yarkovsky Effect by Radar Ranging to Asteroid 6489 Golevka. Science, 302, 1739-1742. https://doi.org/10.1126/science.1091452</t>
+          <t>[1] Gavrik, Y. A., Gavrik, A. L., &amp; Smyslov, A. A. (2016). Distribution of the surface radio brightness of asteroid Golevka constructed from the radar data. Journal of Communications Technology and Electronics, 61, 1347-1353. https://link.springer.com/article/10.1134/S106422691612007X [2] Greenberg, A. H., Margot, J. L., Verma, A. K., Taylor, P. A., &amp; Hodge, S. E. (2020). Yarkovsky Drift Detections for 247 Near-Earth Asteroids. The Astronomical Journal, 159, 92. https://doi.org/10.3847/1538-3881/ab62a3 [3] Hudson, R. S., et al. (2000). Asteroid radar shape models: 6489 Golevka. Planetary Data System, 11, 7. https://ui.adsabs.harvard.edu/abs/2000PDSS...11....7H/abstract [4] Nolan, M. C., et al. (2000). Asteroid radar shape models. Planetary Data System, 11. https://ui.adsabs.harvard.edu/abs/2000PDSS...11.....N/abstract [5] Hudson, R. S., Ostro, S. J., Jurgens, R. F., Rosema, K. D., Giorgini, J. D., Winkler, R., Rose, R., Choate, D., Cormier, R. A., Franck, C. R., Frye, R., Howard, D., Kelley, D., Littlefair, R., Slade, M. A., Benner, L. A. M., Thomas, M. L., Mitchell, D. L., Chodas, P. W., Yeomans, D. K., Scheeres, D. J., Palmer, P., Zaitsev, A., Koyama, Y., Nakamura, A., Harris, A. W., &amp; Meshkov, M. N. (2000). Radar Observations and Physical Model of Asteroid 6489 Golevka. Icarus, 148, 37-51. https://doi.org/10.1006/icar.2000.6483 [6] Koyama, Y., Nakajima, J., Sekido, M., Yoshikawa, M., Nakamura, A. M., Hirabayashi, H., Okada, T., Abe, M., Nishibori, T., Fuse, T., Ostro, S. J., Choate, D., Cormier, R. A., Winkler, R., Jurgens, R. F., Giorgini, J. D., Yeomans, D. K., Slade, M. A., &amp; Zaitsev, A. L. (2001). Radar observations of near-Earth asteroids 6489 Golevka and 4197 (1982 TA). Communications Research Laboratory Review, 47, 145. https://ui.adsabs.harvard.edu/abs/2001CRLRv..47..145K/abstract [7] Zaitsev, A. L., Ostro, S. J., Ignatov, S. M., Yeomans, D. K., Petrenko, B. L., Choate, D., Margorin, O. K., Cormier, R. A., Mardyshkin, V. P., Winkler, R., Rghiga, D., Jurgens, R. F., Shubin, K. L., Giorgini, J. D., Krivtsov, A. P., Rosema, K. D., Koluka, Y. F., Slade, M. A., Gavrik, A. L., Andreev, O. N., Ivanov, A. E., Peshin, S. V., Koyama, Y., Yoshikawa, M., &amp; Nakamura, A. (1997). Intercontinental bistatic radar observations of 6489 Golevka (1991 JX). Planetary and Space Science, 45, 771-778. https://doi.org/10.1016/S0032-0633(97)00042-1 [8] Chesley, S. R., Ostro, S. J., Vokrouhlický, D., Čapek, D., Giorgini, J. D., Nolan, M. C., Margot, J. L., Hine, A. A., Benner, L. A. M., &amp; Chamberlin, A. B. (2003). Direct Detection of the Yarkovsky Effect by Radar Ranging to Asteroid 6489 Golevka. Science, 302, 1739-1742. https://doi.org/10.1126/science.1091452</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -4930,7 +4930,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>[1] (2012). (. , 3176, 1. https://ui.adsabs.harvard.edu/abs/2012CBET.3176....1T/abstract</t>
+          <t>[1] (2012). (5143) Heracles. Central Bureau Electronic Telegrams, 3176. https://ui.adsabs.harvard.edu/abs/2012CBET.3176....1T/abstract</t>
         </is>
       </c>
       <c r="P66" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>[1] (2004). R. , 36, 32.29. https://ui.adsabs.harvard.edu/abs/2004DPS....36.3229B/abstract [2] (2012). R. , 44, 302.05. https://ui.adsabs.harvard.edu/abs/2012DPS....4430205B/abstract</t>
+          <t>[1] Benner, L. A. M., Nolan, M. C., Carter, L. M., Ostro, S. J., Giorgini, J. D., Magri, C., &amp; Margot, J. L. (2004). Radar imaging of near-Earth asteroid 11066 Sigurd. AAS/DPS Meeting #36, 32.29. https://ui.adsabs.harvard.edu/abs/2004DPS....36.3229B/abstract [2] Busch, M. W., et al. (2012). Radar Imaging Of 11066 Sigurd, 2000 YF29, And 2004 XL14 And The Obliquity Distribution Of Contact Binary Near-Earth Asteroids. AAS/DPS Meeting #44, 302.05. https://ui.adsabs.harvard.edu/abs/2012DPS....4430205B/abstract</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -5715,7 +5715,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>[1] (2014). T. , 46, 409.03. https://ui.adsabs.harvard.edu/abs/2014DPS....4640903T/abstract</t>
+          <t>[1] Taylor, P. A., et al. (2014). The Smallest Binary Asteroid? The Discovery of Equal-Mass Binary 1994 CJ1. AAS/DPS Meeting #46, 409.03. https://ui.adsabs.harvard.edu/abs/2014DPS....4640903T/abstract</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
@@ -6105,7 +6105,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>[1] (2005). 1. , 8563, 2. https://ui.adsabs.harvard.edu/abs/2005IAUC.8563....2B/abstract</t>
+          <t>[1] Benner, L. A. M., Nolan, M. C., Ostro, S. J., Giorgini, J. D., Margot, J. L., &amp; Magri, C. (2005). 1994 XD. IAU Circular, 8563. https://ui.adsabs.harvard.edu/abs/2005IAUC.8563....2B/abstract</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>[1] (2012). A. , 1667, 6403. https://ui.adsabs.harvard.edu/abs/2012LPICo1667.6403B/abstract [2] (2012). 1. , EPSC2012-542. https://ui.adsabs.harvard.edu/abs/2012epsc.conf..542C/abstract</t>
+          <t>[1] Benner, L. A. M., et al. (2012). Radar Observations of Near-Earth Asteroid (175706) 1996 FG3. Lunar and Planetary Institute Contributions, 1667, 6403. https://ui.adsabs.harvard.edu/abs/2012LPICo1667.6403B/abstract [2] (2012). 1996 FG3, MarcoPolo-R mission target: Living on the edge. EPSC Abstracts, 7, 542. https://ui.adsabs.harvard.edu/abs/2012epsc.conf..542C/abstract</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
@@ -6445,7 +6445,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>[1] (2020). R. , 348, 113777. https://doi.org/10.1016/j.icarus.2020.113777 [2] (2010). R. , 42, 13.17. https://ui.adsabs.harvard.edu/abs/2010DPS....42.1317B/abstract [3] (2022). A. , 3, 210. https://doi.org/10.3847/PSJ/ac880d [4] (2016). O. , P52B-02. https://ui.adsabs.harvard.edu/abs/2016AGUFM.P52B..02N/abstract [5] (2003). (. , 8244, 2. https://ui.adsabs.harvard.edu/abs/2003IAUC.8244....2P/abstract [6] Pajola, M., Barnouin, O. S., Lucchetti, A., Hirabayashi, M., Ballouz, R.-L., Asphaug, E., Ernst, C. M., Della Corte, V., Farnham, T., Poggiali, G., Sunshine, J. M., Epifani, E. M., Murdoch, N., Ieva, S., Schwartz, S. R., Ivanovski, S., Trigo-Rodriguez, J. M., Rossi, A., Chabot, N. L., Zinzi, A., Rivkin, A., Brucato, J. R., Michel, P., Cremonese, G., Dotto, E., Amoroso, M., Bertini, I., Capannolo, A., Cheng, A., Cotugno, B., Dall'Ora, M., Daly, R. T., Di Tana, V., Deshapriya, J. D. P., Gai, I., Hasselmann, P. H. A., Impresario, G., Lavagna, M., Meneghin, A., Miglioretti, F., Modenini, D., Palumbo, P., Perna, D., Pirrotta, S., Simioni, E., Simonetti, S., Tortora, P., Zannoni, M., and Zanotti, G., Anticipated Geological Assessment of the (65803) Didymos-Dimorphos System, Target of the DART-LICIACube Mission, The Planetary Science Journal, 3, p.210, 2022 https://ui.adsabs.harvard.edu/abs/2022PSJ.....3..210P</t>
+          <t>[1] Naidu, S.P., Benner, L.A.M., Brozovic, M., Nolan, M.C., Ostro, S.J., Margot, J.L., Giorgini, J.D., &amp; Hirabayashi, T. (2020). Radar observations and a physical model of binary near-Earth asteroid 65803 Didymos, target of the DART mission. Icarus, 348, 113777. https://doi.org/10.1016/j.icarus.2020.113777 [2] Benner, L. A. M., et al. (2010). Radar Imaging and a Physical Model of Binary Asteroid 65803 Didymos. AAS/DPS Meeting #42, 13.17. https://ui.adsabs.harvard.edu/abs/2010DPS....42.1317B/abstract [3] Pajola, M., Barnouin, O.S., Lucchetti, A., Hirabayashi, M., Ballouz, R.-L., Asphaug, E., Ernst, C.M., &amp; Della Corte, V. (2022). Anticipated Geological Assessment of the (65803) Didymos-Dimorphos System, Target of the DART-LICIACube Mission. The Planetary Science Journal, 3, 210. https://doi.org/10.3847/PSJ/ac880d [4] Naidu, S. P., et al. (2016). Radar observations of binary near-Earth asteroid 65803 Didymos. AGU Fall Meeting, abstract P52B-02. https://ui.adsabs.harvard.edu/abs/2016AGUFM.P52B..02N/abstract [5] (2003). 65803 Didymos (1996 GT). IAU Circular, 8244. https://ui.adsabs.harvard.edu/abs/2003IAUC.8244....2P/abstract [6] Pajola, M., Barnouin, O. S., Lucchetti, A., Hirabayashi, M., Ballouz, R.-L., Asphaug, E., Ernst, C. M., Della Corte, V., Farnham, T., Poggiali, G., Sunshine, J. M., Epifani, E. M., Murdoch, N., Ieva, S., Schwartz, S. R., Ivanovski, S., Trigo-Rodriguez, J. M., Rossi, A., Chabot, N. L., Zinzi, A., Rivkin, A., Brucato, J. R., Michel, P., Cremonese, G., Dotto, E., Amoroso, M., Bertini, I., Capannolo, A., Cheng, A., Cotugno, B., Dall'Ora, M., Daly, R. T., Di Tana, V., Deshapriya, J. D. P., Gai, I., Hasselmann, P. H. A., Impresario, G., Lavagna, M., Meneghin, A., Miglioretti, F., Modenini, D., Palumbo, P., Perna, D., Pirrotta, S., Simioni, E., Simonetti, S., Tortora, P., Zannoni, M., and Zanotti, G., Anticipated Geological Assessment of the (65803) Didymos-Dimorphos System, Target of the DART-LICIACube Mission, The Planetary Science Journal, 3, p.210, 2022 https://ui.adsabs.harvard.edu/abs/2022PSJ.....3..210P</t>
         </is>
       </c>
       <c r="P89" t="inlineStr">
@@ -7130,7 +7130,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>[1] (2009). A. , 41, 43.09. https://ui.adsabs.harvard.edu/abs/2009DPS....41.4309B/abstract</t>
+          <t>[1] Benner, L. A. M., et al. (2009). Radar Imaging of Near-Earth Asteroid 1998 CS1. AAS/DPS Meeting #41, 43.09. https://ui.adsabs.harvard.edu/abs/2009DPS....41.4309B/abstract</t>
         </is>
       </c>
       <c r="P99" t="inlineStr">
@@ -8020,7 +8020,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>[1] (2003). (. , 8216, 3. https://ui.adsabs.harvard.edu/abs/2003IAUC.8216....3P/abstract</t>
+          <t>[1] (2003). (66063) 1998 RO1. IAU Circular, 8216. https://ui.adsabs.harvard.edu/abs/2003IAUC.8216....3P/abstract</t>
         </is>
       </c>
       <c r="P112" t="inlineStr">
@@ -8365,7 +8365,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>[1] (2003). R. , 35, 24.01. https://ui.adsabs.harvard.edu/abs/2003DPS....35.2401B/abstract</t>
+          <t>[1] Benner, L. A. M., et al. (2003). Radar Imaging of Binary Near-Earth Asteroid 1998 ST27. AAS/DPS Meeting #35, 24.01. https://ui.adsabs.harvard.edu/abs/2003DPS....35.2401B/abstract</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -9580,7 +9580,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>[1] (2013). P. , 5132, 1. https://ui.adsabs.harvard.edu/abs/2013ATel.5132....1H/abstract</t>
+          <t>[1] Hicks, M., et al. (2013). Palomar Spectroscopy of Near-Earth Asteroids 137199 (1999 KX4), 152756 (1999 JV3), 163249 (2002 GT), 163364 (2002 OD20), and 285263 (1998 QE2). The Astronomer's Telegram, 5132. http://www.astronomerstelegram.org/?read=5132</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
@@ -9815,7 +9815,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>[1] (2013). P. , 5132, 1. https://ui.adsabs.harvard.edu/abs/2013ATel.5132....1H/abstract</t>
+          <t>[1] Hicks, M., et al. (2013). Palomar Spectroscopy of Near-Earth Asteroids 137199 (1999 KX4), 152756 (1999 JV3), 163249 (2002 GT), 163364 (2002 OD20), and 285263 (1998 QE2). The Astronomer's Telegram, 5132. http://www.astronomerstelegram.org/?read=5132</t>
         </is>
       </c>
       <c r="P138" t="inlineStr">
@@ -9925,7 +9925,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>[1] (2010). B. , 2706, 1. https://ui.adsabs.harvard.edu/abs/2010ATel.2706....1H/abstract</t>
+          <t>[1] Hicks, M., et al. (2010). Broadband Photometry of the Potentially Hazardous Asteroid 1999 MN: Suggestive of YORP and/or Tidal Spin-Up?. The Astronomer's Telegram, 2706. http://www.astronomerstelegram.org/?read=2706</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
@@ -10555,7 +10555,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>[1] (2020). (. , 4787, 1. https://ui.adsabs.harvard.edu/abs/2020CBET.4787....1G/abstract</t>
+          <t>[1] (2020). (264357) 2000 AZ_93. Central Bureau Electronic Telegrams, 4787. https://ui.adsabs.harvard.edu/abs/2020CBET.4787....1G/abstract</t>
         </is>
       </c>
       <c r="P150" t="inlineStr">
@@ -10835,7 +10835,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>[1] (2010). R. , 42, 13.18. https://ui.adsabs.harvard.edu/abs/2010DPS....42.1318J/abstract</t>
+          <t>[1] Jimenez, A., et al. (2010). Radar Shape Modeling of Binary Near-Earth Asteroid 2000 CO101. AAS/DPS Meeting #42, 13.18. https://ui.adsabs.harvard.edu/abs/2010DPS....42.1318J/abstract</t>
         </is>
       </c>
       <c r="P154" t="inlineStr">
@@ -11355,7 +11355,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>[1] (2012). T. , 44, 111.10. https://ui.adsabs.harvard.edu/abs/2012DPS....4411110V/abstract [2] (2013). R. , 226, 323. https://doi.org/10.1016/j.icarus.2013.05.025 [3] (2012). R. , 44, 302.06. https://ui.adsabs.harvard.edu/abs/2012DPS....4430206N/abstract [4] Marshall, S.E., E.S. Howell, C. Magri, R.J. Vervack, D.B. Campbell, Y.R. Fernandez, M.C. Nolan, J.L. Crowell, M.D. Hicks, K.J. Lawrence, and P.A. Taylor, Thermal Properties and an Improved Shape Model for Near-Earth Asteroid (162421) 2000 ET70, Icarus 292, 22-35, 2017 http://dx.doi.org/10.1016/j.icarus.2017.03.028</t>
+          <t>[1] (2012). The Asteroid 2000 ET70. AAS/DPS Meeting #44, 111.10. https://ui.adsabs.harvard.edu/abs/2012DPS....4411110V/abstract [2] Naidu, S.P., Margot, J.L., Busch, M.W., Taylor, P.A., Nolan, M.C., Brozovic, M., Benner, L.A.M., &amp; Giorgini, J.D. (2013). Radar imaging and physical characterization of near-Earth Asteroid (162421) 2000 ET70. Icarus, 226, 323-335. https://doi.org/10.1016/j.icarus.2013.05.025 [3] Naidu, S. P., &amp; Margot, J. L. (2012). Radar Imaging and Physical Characterization of Near-Earth Asteroid (162421) 2000 ET70. AAS/DPS Meeting #44, 302.06. https://ui.adsabs.harvard.edu/abs/2012DPS....4430206N/abstract [4] Marshall, S.E., E.S. Howell, C. Magri, R.J. Vervack, D.B. Campbell, Y.R. Fernandez, M.C. Nolan, J.L. Crowell, M.D. Hicks, K.J. Lawrence, and P.A. Taylor, Thermal Properties and an Improved Shape Model for Near-Earth Asteroid (162421) 2000 ET70, Icarus 292, 22-35, 2017 http://dx.doi.org/10.1016/j.icarus.2017.03.028</t>
         </is>
       </c>
       <c r="P162" t="inlineStr">
@@ -12170,7 +12170,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>[1] (2009). P. , 2323, 1. https://ui.adsabs.harvard.edu/abs/2009ATel.2323....1H/abstract [2] (2009). L. , 2283, 1. https://ui.adsabs.harvard.edu/abs/2009ATel.2283....1H/abstract</t>
+          <t>[1] Hicks, M., et al. (2009). Planetary radar targets 1999 AP10, 2000 TO64, 2000 UJ1, and 2000 XK44: Four S-complex near-Earth asteroids. The Astronomer's Telegram, 2323. http://www.astronomerstelegram.org/?read=2323</t>
         </is>
       </c>
       <c r="P175" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>[1] (2001). R. , 2055. https://ui.adsabs.harvard.edu/abs/2001LPI....32.2055N/abstract</t>
+          <t>[1] Nolan, M. C., Margot, J. L., Howell, E. S., &amp; Benner, L. A. M. (2001). Radar Observations of Near-Earth Asteroids 2000 UG11 and 2000 UK11. Lunar and Planetary Science Conference, 32, 2055. https://ui.adsabs.harvard.edu/abs/2001LPI....32.2055N/abstract</t>
         </is>
       </c>
       <c r="P176" t="inlineStr">
@@ -12290,7 +12290,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>[1] (2009). P. , 2323, 1. https://ui.adsabs.harvard.edu/abs/2009ATel.2323....1H/abstract [2] (2009). L. , 2283, 1. https://ui.adsabs.harvard.edu/abs/2009ATel.2283....1H/abstract</t>
+          <t>[1] Hicks, M., et al. (2009). Planetary radar targets 1999 AP10, 2000 TO64, 2000 UJ1, and 2000 XK44: Four S-complex near-Earth asteroids. The Astronomer's Telegram, 2323. http://www.astronomerstelegram.org/?read=2323</t>
         </is>
       </c>
       <c r="P177" t="inlineStr">
@@ -12340,7 +12340,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>[1] (2001). R. , 2055. https://ui.adsabs.harvard.edu/abs/2001LPI....32.2055N/abstract</t>
+          <t>[1] Nolan, M. C., Margot, J. L., Howell, E. S., &amp; Benner, L. A. M. (2001). Radar Observations of Near-Earth Asteroids 2000 UG11 and 2000 UK11. Lunar and Planetary Science Conference, 32, 2055. https://ui.adsabs.harvard.edu/abs/2001LPI....32.2055N/abstract</t>
         </is>
       </c>
       <c r="P178" t="inlineStr">
@@ -12400,7 +12400,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>[1] (2009). P. , 2323, 1. https://ui.adsabs.harvard.edu/abs/2009ATel.2323....1H/abstract [2] (2010). 2. , 2371, 1. https://ui.adsabs.harvard.edu/abs/2010ATel.2371....1H/abstract</t>
+          <t>[1] Hicks, M., et al. (2009). Planetary radar targets 1999 AP10, 2000 TO64, 2000 UJ1, and 2000 XK44: Four S-complex near-Earth asteroids. The Astronomer's Telegram, 2323. http://www.astronomerstelegram.org/?read=2323</t>
         </is>
       </c>
       <c r="P179" t="inlineStr">
@@ -12570,7 +12570,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>[1] (2012). R. , 44, 302.05. https://ui.adsabs.harvard.edu/abs/2012DPS....4430205B/abstract</t>
+          <t>[1] Busch, M. W., et al. (2012). Radar Imaging Of 11066 Sigurd, 2000 YF29, And 2004 XL14 And The Obliquity Distribution Of Contact Binary Near-Earth Asteroids. AAS/DPS Meeting #44, 302.05. https://ui.adsabs.harvard.edu/abs/2012DPS....4430205B/abstract</t>
         </is>
       </c>
       <c r="P182" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>[1] (2010). P. , 2502, 1. https://ui.adsabs.harvard.edu/abs/2010ATel.2502....1H/abstract</t>
+          <t>[1] Hicks, M., et al. (2010). Physical Characterization of the Potentially Hazardous Asteroid and Planetary Radar Target 68216 (2001 CV26): An Excellent Shape/Pole Modeling Candidate. The Astronomer's Telegram, 2502. http://www.astronomerstelegram.org/?read=2502</t>
         </is>
       </c>
       <c r="P190" t="inlineStr">
@@ -14720,7 +14720,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>[1] (2021). C. , 95. https://ui.adsabs.harvard.edu/abs/2021plde.confE..95T/abstract</t>
+          <t>[1] Taylor, P. A., et al. (2021). Characterization of Near-Earth Asteroid 153814 (2001 WN5) and Prospects for the 2028 Close Encounter with Earth. 7th IAA Planetary Defense Conference, E-95. https://ui.adsabs.harvard.edu/abs/2021plde.confE..95T/abstract</t>
         </is>
       </c>
       <c r="P218" t="inlineStr">
@@ -15230,7 +15230,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>[1] (2013). P. , 45, 208.08. https://ui.adsabs.harvard.edu/abs/2013DPS....4520808T/abstract</t>
+          <t>[1] Taylor, P. A., et al. (2013). Physical Characterization of Binary Near-Earth Asteroid (153958) 2002 AM31. AAS/DPS Meeting #45, 208.08. https://ui.adsabs.harvard.edu/abs/2013DPS....4520808T/abstract</t>
         </is>
       </c>
       <c r="P227" t="inlineStr">
@@ -17855,7 +17855,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>[1] (2014). B. , 6090, 1. https://ui.adsabs.harvard.edu/abs/2014ATel.6090....1H/abstract</t>
+          <t>[1] Hicks, M., et al. (2014). Broad-band photometry of NHATS target 387733 (2003 GS). The Astronomer's Telegram, 6090. http://www.astronomerstelegram.org/?read=6090</t>
         </is>
       </c>
       <c r="P270" t="inlineStr">
@@ -18765,7 +18765,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>[1] (2021). (. , 5037, 1. https://ui.adsabs.harvard.edu/abs/2021CBET.5037....1P/abstract</t>
+          <t>[1] (2021). (143649) 2003 QQ_47. Central Bureau Electronic Telegrams, 5037. https://ui.adsabs.harvard.edu/abs/2021CBET.5037....1P/abstract</t>
         </is>
       </c>
       <c r="P285" t="inlineStr">
@@ -19340,7 +19340,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>[1] (2017). (. , 4353, 1. https://ui.adsabs.harvard.edu/abs/2017CBET.4353....1B/abstract</t>
+          <t>[1] (2017). (226514) 2003 UX_34. Central Bureau Electronic Telegrams, 4353. https://ui.adsabs.harvard.edu/abs/2017CBET.4353....1B/abstract</t>
         </is>
       </c>
       <c r="P294" t="inlineStr">
@@ -19875,7 +19875,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>[1] (2004). R. , 36, 28.08. https://ui.adsabs.harvard.edu/abs/2004DPS....36.2808N/abstract [2] (2004). C. , 36, 28.09. https://ui.adsabs.harvard.edu/abs/2004DPS....36.2809A/abstract [3] (2009). B. , 2289, 1. https://ui.adsabs.harvard.edu/abs/2009ATel.2289....1H/abstract</t>
+          <t>[1] Nolan, M. C., et al. (2004). Radar Images of Binary Asteroid 2003 YT1. AAS/DPS Meeting #36, 28.08. https://ui.adsabs.harvard.edu/abs/2004DPS....36.2808N/abstract [2] (2004). Compositional Results of Binary Near-Earth Asteroid 2003 YT1: A Basaltic Achondrite. AAS/DPS Meeting #36, 28.09. https://ui.adsabs.harvard.edu/abs/2004DPS....36.2809A/abstract [3] Hicks, M., et al. (2009). Broad-band Photometry of the Binary Potentially Hazardous Asteroid 2003 YT1. The Astronomer's Telegram, 2289. http://www.astronomerstelegram.org/?read=2289</t>
         </is>
       </c>
       <c r="P302" t="inlineStr">
@@ -20050,7 +20050,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>[1] (2015). R. , 29, 2257549. https://ui.adsabs.harvard.edu/abs/2015IAUGA..2257549B/abstract</t>
+          <t>[1] Benner, L. A. M., et al. (2015). Radar Imaging of Binary Near-Earth Asteroid (357439) 2004 BL86. IAU General Assembly, 22, 57549. https://ui.adsabs.harvard.edu/abs/2015IAUGA..2257549B/abstract</t>
         </is>
       </c>
       <c r="P305" t="inlineStr">
@@ -20200,7 +20200,7 @@
       </c>
       <c r="O307" t="inlineStr">
         <is>
-          <t>[1] (2006). 2. , 535, 1. https://ui.adsabs.harvard.edu/abs/2006CBET..535....1T/abstract [2] (2006). R. , 38, 50.04. https://ui.adsabs.harvard.edu/abs/2006DPS....38.5004T/abstract</t>
+          <t>[1] (2006). 2004 DC. Central Bureau Electronic Telegrams, 535. https://ui.adsabs.harvard.edu/abs/2006CBET..535....1T/abstract [2] Taylor, P. A., Margot, J. L., Nolan, M. C., Benner, L. A. M., Ostro, S. J., Giorgini, J. D., &amp; Magri, C. (2006). Radar imaging of binary near-Earth Asteroid 2004 DC. Bulletin of the American Astronomical Society, 38, 577. https://ui.adsabs.harvard.edu/abs/2006DPS....38.5004T/abstract</t>
         </is>
       </c>
       <c r="P307" t="inlineStr">
@@ -20420,7 +20420,7 @@
       </c>
       <c r="O310" t="inlineStr">
         <is>
-          <t>[1] (2012). 2. , 3091, 1. https://ui.adsabs.harvard.edu/abs/2012CBET.3091....1T/abstract</t>
+          <t>[1] (2012). 2004 FG11. Central Bureau Electronic Telegrams, 3091. https://ui.adsabs.harvard.edu/abs/2012CBET.3091....1T/abstract</t>
         </is>
       </c>
       <c r="P310" t="inlineStr">
@@ -21690,7 +21690,7 @@
       </c>
       <c r="O331" t="inlineStr">
         <is>
-          <t>[1] (2012). R. , 44, 302.05. https://ui.adsabs.harvard.edu/abs/2012DPS....4430205B/abstract</t>
+          <t>[1] Busch, M. W., et al. (2012). Radar Imaging Of 11066 Sigurd, 2000 YF29, And 2004 XL14 And The Obliquity Distribution Of Contact Binary Near-Earth Asteroids. AAS/DPS Meeting #44, 302.05. https://ui.adsabs.harvard.edu/abs/2012DPS....4430205B/abstract</t>
         </is>
       </c>
       <c r="P331" t="inlineStr">
@@ -24080,7 +24080,7 @@
       </c>
       <c r="O371" t="inlineStr">
         <is>
-          <t>[1] (2011). Preparing for asteroid 2005 YU55 at close quarters. Astronomy &amp;amp; Geophysics, 52, 3.06-3.06. https://doi.org/10.1111/j.1468-4004.2011.52304_10.x [2] Vereshchagina, I. A., Sokov, E. N., Gorshanov, D. L., Devyatkin, A. V., L’vov, V. N., Tsekmeister, S. D., Romas, E. S., &amp; Martyusheva, A. A. (2014). Astrometry and photometry of asteroid (308635) 2005 YU55. Solar System Research, 48, 382-390. https://doi.org/10.1134/s0038094614040108</t>
+          <t>[1] (2011). Preparing for asteroid 2005 YU55 at close quarters. Astronomy &amp; Geophysics, 52, 3.06. https://doi.org/10.1111/j.1468-4004.2011.52304_10.x [2] Vereshchagina, I. A., Sokov, E. N., Gorshanov, D. L., Devyatkin, A. V., L’vov, V. N., Tsekmeister, S. D., Romas, E. S., &amp; Martyusheva, A. A. (2014). Astrometry and photometry of asteroid (308635) 2005 YU55. Solar System Research, 48, 382-390. https://doi.org/10.1134/s0038094614040108</t>
         </is>
       </c>
       <c r="P371" t="inlineStr">
@@ -24510,7 +24510,7 @@
       </c>
       <c r="O378" t="inlineStr">
         <is>
-          <t>[1] (2006). 2. , 534, 1. https://ui.adsabs.harvard.edu/abs/2006CBET..534....1B/abstract</t>
+          <t>[1] (2006). 2006 GY2. Central Bureau Electronic Telegrams, 534. https://ui.adsabs.harvard.edu/abs/2006CBET..534....1B/abstract</t>
         </is>
       </c>
       <c r="P378" t="inlineStr">
@@ -25170,7 +25170,7 @@
       </c>
       <c r="O389" t="inlineStr">
         <is>
-          <t>[1] (2025). L. , 52, 100. https://ui.adsabs.harvard.edu/abs/2025MPBu...52..100N/abstract</t>
+          <t>[1] (2025). Lightcurve Analysis and Rotation Period for NEA 2006 WB. Minor Planet Bulletin, 52, 100. https://ui.adsabs.harvard.edu/abs/2025MPBu...52..100N/abstract</t>
         </is>
       </c>
       <c r="P389" t="inlineStr">
@@ -27325,7 +27325,7 @@
       </c>
       <c r="O424" t="inlineStr">
         <is>
-          <t>[1] (2017). S. , 230, 119.01. https://ui.adsabs.harvard.edu/abs/2017AAS...23011901V/abstract</t>
+          <t>[1] Quijano Vodniza, A. (2017). Study of the Asteroid 2009 DL46. AAS Meeting #230, 119.01. https://ui.adsabs.harvard.edu/abs/2017AAS...23011901V/abstract</t>
         </is>
       </c>
       <c r="P424" t="inlineStr">
@@ -28975,7 +28975,7 @@
       </c>
       <c r="O449" t="inlineStr">
         <is>
-          <t>[1] (2016). (. , 4304, 1. https://ui.adsabs.harvard.edu/abs/2016CBET.4304....1G/abstract</t>
+          <t>[1] (2016). (441987) 2010 NY_65. Central Bureau Electronic Telegrams, 4304. https://ui.adsabs.harvard.edu/abs/2016CBET.4304....1G/abstract</t>
         </is>
       </c>
       <c r="P449" t="inlineStr">
@@ -37220,7 +37220,7 @@
       </c>
       <c r="O597" t="inlineStr">
         <is>
-          <t>[1] (2020). 2. , 4786, 1. https://ui.adsabs.harvard.edu/abs/2020CBET.4786....1G/abstract</t>
+          <t>[1] (2020). 2015 EG. Central Bureau Electronic Telegrams, 4786. https://ui.adsabs.harvard.edu/abs/2020CBET.4786....1G/abstract</t>
         </is>
       </c>
       <c r="P597" t="inlineStr">
@@ -37675,7 +37675,7 @@
       </c>
       <c r="O605" t="inlineStr">
         <is>
-          <t>[1] (2015). A. , 47, 402.05. https://ui.adsabs.harvard.edu/abs/2015DPS....4740205B/abstract</t>
+          <t>[1] (2015). Asteroids With Tensile Strength: The Case of 2015 HM10. AAS/DPS Meeting #47, 402.05. https://ui.adsabs.harvard.edu/abs/2015DPS....4740205B/abstract</t>
         </is>
       </c>
       <c r="P605" t="inlineStr">
@@ -39075,7 +39075,7 @@
       </c>
       <c r="O629" t="inlineStr">
         <is>
-          <t>[1] Müller, T. G., Marciniak, A., Butkiewicz-Bąk, M., Duffard, R., Oszkiewicz, D., Käufl, H. U., Szakáts, R., Santana-Ros, T., Kiss, C., &amp; Santos-Sanz, P. (2017). Large Halloween asteroid at lunar distance. Astronomy &amp;amp; Astrophysics, 598, A63. https://doi.org/10.1051/0004-6361/201629584 [2] R. et al. (2016). Bulletin of the American Astronomical Society (DPS meeting abstract), Vol. 4832910. [ADS record] https://ui.adsabs.harvard.edu/abs/2016DPS....4832910R/abstract [3] Busch, M. W., et al. (2016). Recent radar observations of potentially hazardous near-Earth asteroids with the Arecibo Observatory and the Deep Space Network. AGU Fall Meeting, abstract NH12A-06. https://ui.adsabs.harvard.edu/abs/2016AGUFMNH12A..06B/abstract</t>
+          <t>[1] Müller, T. G., Marciniak, A., Butkiewicz-Bąk, M., Duffard, R., Oszkiewicz, D., Käufl, H. U., Szakáts, R., Santana-Ros, T., Kiss, C., &amp; Santos-Sanz, P. (2017). Large Halloween asteroid at lunar distance. Astronomy &amp;amp; Astrophysics, 598, A63. https://doi.org/10.1051/0004-6361/201629584 [2] Rivera-Valentin, E. G., et al. (2016). Radar observations of near-Earth asteroids from Arecibo Observatory. AAS/DPS Meeting #48, 329.10. https://ui.adsabs.harvard.edu/abs/2016DPS....4832910R/abstract [3] Busch, M. W., et al. (2016). Recent radar observations of potentially hazardous near-Earth asteroids with the Arecibo Observatory and the Deep Space Network. AGU Fall Meeting, abstract NH12A-06. https://ui.adsabs.harvard.edu/abs/2016AGUFMNH12A..06B/abstract</t>
         </is>
       </c>
       <c r="P629" t="inlineStr">
@@ -44295,7 +44295,7 @@
       </c>
       <c r="O727" t="inlineStr">
         <is>
-          <t>[1] (2024). R. , 5, 123. https://doi.org/10.3847/PSJ/ad4342</t>
+          <t>[1] Brozovic, M., Benner, L.A.M., Naidu, S.P., Moskovitz, N., Giorgini, J.D., Virkki, A.K., Marshall, S.E., &amp; Dover, L.R. (2024). Radar and Optical Observations and Physical Modeling of Binary Near-Earth Asteroid 2018 EB. The Planetary Science Journal, 5, 123. https://doi.org/10.3847/PSJ/ad4342</t>
         </is>
       </c>
       <c r="P727" t="inlineStr">
@@ -49960,7 +49960,7 @@
       </c>
       <c r="O837" t="inlineStr">
         <is>
-          <t>[1] (2021). 2. , 53, 207.01. https://ui.adsabs.harvard.edu/abs/2021DPS....5320701Z/abstract</t>
+          <t>[1] Zambrano-Marin, L. F., Marshall, S. E., Howell, E. S., de León, J., Pinilla-Alonso, N., Virkki, A. K., Giorgini, J., &amp; Venditti, F. C. F. (2025). 2020 BX12-The Last Binary Asteroid Discovered at Arecibo. The Planetary Science Journal, 6, 91. https://doi.org/10.3847/PSJ/adbe39</t>
         </is>
       </c>
       <c r="P837" t="inlineStr">
@@ -51420,7 +51420,7 @@
       </c>
       <c r="O866" t="inlineStr">
         <is>
-          <t>[1] (2020). A. , 52, 512.07. https://ui.adsabs.harvard.edu/abs/2020DPS....5251207V/abstract</t>
+          <t>[1] Venditti, F., Marshall, S., Virkki, A., Taylor, P., Hickson, D., &amp; Giorgini, J. (2020). Arecibo Observatory radar observation of potentially hazardous asteroid 2020 NK1. AAS/DPS Meeting #52, 512.07. https://ui.adsabs.harvard.edu/abs/2020DPS....5251207V/abstract</t>
         </is>
       </c>
       <c r="P866" t="inlineStr">
@@ -52310,7 +52310,7 @@
       </c>
       <c r="O883" t="inlineStr">
         <is>
-          <t>[1] (1997). T. , 114, 402. https://doi.org/10.1086/118484</t>
+          <t>[1] Hilton, J.L. (1997). The Mass of the Asteroid 15 Eunomia From Observations of 1313 Berna and 1284 Latvia. The Astronomical Journal, 114, 402. https://doi.org/10.1086/118484</t>
         </is>
       </c>
       <c r="P883" t="inlineStr">
@@ -52945,7 +52945,7 @@
       </c>
       <c r="O894" t="inlineStr">
         <is>
-          <t>[1] (2008). R. , 195, 220. https://doi.org/10.1016/j.icarus.2007.12.018 [2] Reddy, V., J.A. Sanchez, W.F. Bottke, A. Thirouin, E.G. Rivera-Valentin, M.S. Kelley, W. Ryan, E.A. Cloutis, S.C. Tegler, E.V. Ryan, P.A. Taylor, J.E. Richardson, N. Moskovitz, and L. Le Corre, Physical Characterization of 2-m Diameter Near-Earth Asteroid 2015 TC25: A Possible Boulder from E-type Asteroid (44) Nysa, Astronomical Journal 152, 162, 2016 http://dx.doi.org/10.3847/0004-6256/152/6/162</t>
+          <t>[1] Shepard, M.K., Kressler, K.M., Clark, B.E., Ockert-Bell, M.E., Nolan, M.C., Howell, E.S., Magri, C., &amp; Giorgini, J.D. (2008). Radar observations of E-class Asteroids 44 Nysa and 434 Hungaria. Icarus, 195, 220-225. https://doi.org/10.1016/j.icarus.2007.12.018 [2] Reddy, V., J.A. Sanchez, W.F. Bottke, A. Thirouin, E.G. Rivera-Valentin, M.S. Kelley, W. Ryan, E.A. Cloutis, S.C. Tegler, E.V. Ryan, P.A. Taylor, J.E. Richardson, N. Moskovitz, and L. Le Corre, Physical Characterization of 2-m Diameter Near-Earth Asteroid 2015 TC25: A Possible Boulder from E-type Asteroid (44) Nysa, Astronomical Journal 152, 162, 2016 http://dx.doi.org/10.3847/0004-6256/152/6/162</t>
         </is>
       </c>
       <c r="P894" t="inlineStr">
@@ -55755,7 +55755,7 @@
       </c>
       <c r="O945" t="inlineStr">
         <is>
-          <t>[1] (1997). P. , 29, 05.08. https://ui.adsabs.harvard.edu/abs/1997DPS....29.0508O/abstract</t>
+          <t>[1] Ostro, S. J., et al. (1997). Radar Observations of 253 Mathilde. AAS/DPS Meeting #29, 05.08. https://ui.adsabs.harvard.edu/abs/1997DPS....29.0508O/abstract</t>
         </is>
       </c>
       <c r="P945" t="inlineStr">
@@ -56905,7 +56905,7 @@
       </c>
       <c r="O966" t="inlineStr">
         <is>
-          <t>[1] Shepard, M. K., Kressler, K. M., Clark, B. E., Ockert-Bell, M. E., Nolan, M. C., Howell, E. S., Magri, C., Giorgini, J. D., Benner, L. A. M., &amp; Ostro, S. J. (2008). Radar observations of E-class Asteroids 44 Nysa and 434 Hungaria. Icarus, 195, 220-225. https://doi.org/10.1016/j.icarus.2007.12.018 [2] Shepard, M. K., Harris, A. W., Taylor, P. A., Clark, B. E., Ockert-Bell, M., Nolan, M. C., Howell, E. S., Magri, C., Giorgini, J. D., &amp; Benner, L. A. M. (2011). Radar observations of Asteroids 64 Angelina and 69 Hesperia. Icarus, 215, 547-551. https://doi.org/10.1016/j.icarus.2011.07.027</t>
+          <t>[1] Shepard, M.K., Kressler, K.M., Clark, B.E., Ockert-Bell, M.E., Nolan, M.C., Howell, E.S., Magri, C., &amp; Giorgini, J.D. (2008). Radar observations of E-class Asteroids 44 Nysa and 434 Hungaria. Icarus, 195, 220-225. https://doi.org/10.1016/j.icarus.2007.12.018 [2] Shepard, M. K., Harris, A. W., Taylor, P. A., Clark, B. E., Ockert-Bell, M., Nolan, M. C., Howell, E. S., Magri, C., Giorgini, J. D., &amp; Benner, L. A. M. (2011). Radar observations of Asteroids 64 Angelina and 69 Hesperia. Icarus, 215, 547-551. https://doi.org/10.1016/j.icarus.2011.07.027</t>
         </is>
       </c>
       <c r="P966" t="inlineStr">
@@ -58385,7 +58385,7 @@
       </c>
       <c r="O993" t="inlineStr">
         <is>
-          <t>[1] (1983). C. , 3832, 1. https://ui.adsabs.harvard.edu/abs/1983IAUC.3832....1W/abstract</t>
+          <t>[1] (1983). Comet Sugano-Saigusa-Fujikawa (1983e). IAU Circular, 3832. https://ui.adsabs.harvard.edu/abs/1983IAUC.3832....1W/abstract</t>
         </is>
       </c>
       <c r="P993" t="inlineStr">

</xml_diff>